<commit_message>
Doc: EC9 Addition, Glossary [WIP] & Stage 2 Update
- Readded EC8 from earlier deletion as EC9 (Experimental validation or quantitative eval)
- Addition of Glossary and Acronyms table for support
- Updated Stage 2 Progress
- Granted Access to Prof. Tan, David Leong, Teh Zhi Wei (THANK YOU GUYS SO MUCH FOR HELPING <3)

- Can't upload all the papers otherwise I'm gonna get copyright struck to kingdom come :(((((
</commit_message>
<xml_diff>
--- a/Reproducible Section/Step 4 - Stage 2 Screening/QCNN_HQCNN_Screening_Stage2_WIP.xlsx
+++ b/Reproducible Section/Step 4 - Stage 2 Screening/QCNN_HQCNN_Screening_Stage2_WIP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User1\Documents\GitHub\SLR\Reproducible Section\Step 4 - Stage 2 Screening\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29A4941B-B09C-4A4D-BD74-30635CD91C17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3060A46-84A0-46FC-AEFC-F0CCC6FB8791}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PRISMA Dashboard" sheetId="1" r:id="rId1"/>
@@ -43,13 +43,53 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={8FFD76D4-7893-40DB-82DF-8E1BEF512ABF}</author>
+    <author>tc={A4251980-DD93-4931-A79F-2208C274FC20}</author>
+    <author>tc={FD33AB07-11EB-4417-BC00-9F6717F8363D}</author>
     <author>tc={A8621180-8332-4067-A5C3-427EEEAA550B}</author>
     <author>tc={5FCB09E3-43CE-4F41-B07E-5555D6847BA9}</author>
+    <author>tc={4C18BE0C-B936-4C12-970B-A1C978A3A429}</author>
     <author>tc={742400F8-FC12-463E-BF7C-44472F707647}</author>
+    <author>tc={AECB7639-3D48-44A5-A023-E6D739E33DBC}</author>
+    <author>tc={49984621-F60C-4B95-B404-A070273AAB9E}</author>
+    <author>tc={D4CD819D-9741-4F3F-B1F1-A9EDE1B95C3D}</author>
     <author>tc={3BCE51DA-E03A-42CE-BCF4-42F3B17B3F4F}</author>
+    <author>tc={6C607B97-DBE1-4B9B-912B-FC5F378C78F8}</author>
+    <author>tc={9B71B6F6-1440-45C7-B9C6-3D3353E0127E}</author>
+    <author>tc={9A96E512-3F53-4A8F-86C6-E13A0AA03D5D}</author>
+    <author>tc={74FC4EA6-7D43-442D-AC4B-3B99C2479B6D}</author>
+    <author>tc={31E0DE7F-8E71-41E9-98C2-32C7133F7B0E}</author>
+    <author>tc={332BDD9A-D5F7-4A8F-BA56-7686D80374CB}</author>
+    <author>tc={F0C16F01-077A-4435-AC9D-36801D87E965}</author>
+    <author>tc={890B958C-615A-4B5C-8D18-10B0C1B52873}</author>
+    <author>tc={C58A61C8-AE69-4687-8BF9-249CAA893C01}</author>
   </authors>
   <commentList>
-    <comment ref="H61" authorId="0" shapeId="0" xr:uid="{A8621180-8332-4067-A5C3-427EEEAA550B}">
+    <comment ref="J26" authorId="0" shapeId="0" xr:uid="{8FFD76D4-7893-40DB-82DF-8E1BEF512ABF}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    It’s Quantum-Inspired through math, not an actual QCNN</t>
+      </text>
+    </comment>
+    <comment ref="J44" authorId="1" shapeId="0" xr:uid="{A4251980-DD93-4931-A79F-2208C274FC20}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Retracted Paper</t>
+      </text>
+    </comment>
+    <comment ref="J45" authorId="2" shapeId="0" xr:uid="{FD33AB07-11EB-4417-BC00-9F6717F8363D}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    MNIST Dataset, potential man paper</t>
+      </text>
+    </comment>
+    <comment ref="H61" authorId="3" shapeId="0" xr:uid="{A8621180-8332-4067-A5C3-427EEEAA550B}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -57,7 +97,7 @@
     If not EC4, then EC9</t>
       </text>
     </comment>
-    <comment ref="H129" authorId="1" shapeId="0" xr:uid="{5FCB09E3-43CE-4F41-B07E-5555D6847BA9}">
+    <comment ref="H129" authorId="4" shapeId="0" xr:uid="{5FCB09E3-43CE-4F41-B07E-5555D6847BA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -65,7 +105,15 @@
     Would also be EC9</t>
       </text>
     </comment>
-    <comment ref="H142" authorId="2" shapeId="0" xr:uid="{742400F8-FC12-463E-BF7C-44472F707647}">
+    <comment ref="J134" authorId="5" shapeId="0" xr:uid="{4C18BE0C-B936-4C12-970B-A1C978A3A429}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Retracted Paper</t>
+      </text>
+    </comment>
+    <comment ref="H142" authorId="6" shapeId="0" xr:uid="{742400F8-FC12-463E-BF7C-44472F707647}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -73,7 +121,31 @@
     EC9 aswell</t>
       </text>
     </comment>
-    <comment ref="H338" authorId="3" shapeId="0" xr:uid="{3BCE51DA-E03A-42CE-BCF4-42F3B17B3F4F}">
+    <comment ref="J188" authorId="7" shapeId="0" xr:uid="{AECB7639-3D48-44A5-A023-E6D739E33DBC}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Mandarin Language</t>
+      </text>
+    </comment>
+    <comment ref="J248" authorId="8" shapeId="0" xr:uid="{49984621-F60C-4B95-B404-A070273AAB9E}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    MNIST Dataset</t>
+      </text>
+    </comment>
+    <comment ref="J291" authorId="9" shapeId="0" xr:uid="{D4CD819D-9741-4F3F-B1F1-A9EDE1B95C3D}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    MNIST Dataset, author acknowledges it</t>
+      </text>
+    </comment>
+    <comment ref="H338" authorId="10" shapeId="0" xr:uid="{3BCE51DA-E03A-42CE-BCF4-42F3B17B3F4F}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -81,12 +153,88 @@
     Would’ve loved to use this paper :(</t>
       </text>
     </comment>
+    <comment ref="J378" authorId="11" shapeId="0" xr:uid="{6C607B97-DBE1-4B9B-912B-FC5F378C78F8}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Tough Case, needs review:
+- Pros:
+Implementation of a QCNN
+- Cons:
+Benchmarking purpose</t>
+      </text>
+    </comment>
+    <comment ref="J380" authorId="12" shapeId="0" xr:uid="{9B71B6F6-1440-45C7-B9C6-3D3353E0127E}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    No QCNN Application</t>
+      </text>
+    </comment>
+    <comment ref="J404" authorId="13" shapeId="0" xr:uid="{9A96E512-3F53-4A8F-86C6-E13A0AA03D5D}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Shouldn’t have been included in stage 1, didn’t know what the Iris dataset was about-</t>
+      </text>
+    </comment>
+    <comment ref="J489" authorId="14" shapeId="0" xr:uid="{74FC4EA6-7D43-442D-AC4B-3B99C2479B6D}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    MNIST &amp; FMNIST Dataset</t>
+      </text>
+    </comment>
+    <comment ref="J502" authorId="15" shapeId="0" xr:uid="{31E0DE7F-8E71-41E9-98C2-32C7133F7B0E}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Review</t>
+      </text>
+    </comment>
+    <comment ref="J513" authorId="16" shapeId="0" xr:uid="{332BDD9A-D5F7-4A8F-BA56-7686D80374CB}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    MNIST, Autonomous Driving is theoretical and not an application</t>
+      </text>
+    </comment>
+    <comment ref="J521" authorId="17" shapeId="0" xr:uid="{F0C16F01-077A-4435-AC9D-36801D87E965}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    MNIST Dataset</t>
+      </text>
+    </comment>
+    <comment ref="J528" authorId="18" shapeId="0" xr:uid="{890B958C-615A-4B5C-8D18-10B0C1B52873}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Good Proposal, only applied against MNIST &amp; FMNIST :(</t>
+      </text>
+    </comment>
+    <comment ref="J547" authorId="19" shapeId="0" xr:uid="{C58A61C8-AE69-4687-8BF9-249CAA893C01}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Could be interpreted as theoretical, but case studies are relevant and applicable(?)</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4523" uniqueCount="2838">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4567" uniqueCount="2844">
   <si>
     <t>IDENTIFICATION</t>
   </si>
@@ -8600,13 +8748,31 @@
   </si>
   <si>
     <t xml:space="preserve">  EC8</t>
+  </si>
+  <si>
+    <t>Passed by Mahmoud</t>
+  </si>
+  <si>
+    <t>EC7 | Needs Review</t>
+  </si>
+  <si>
+    <t>EC7 | Need Review</t>
+  </si>
+  <si>
+    <t>Passed by Mahmoud | Needs Review</t>
+  </si>
+  <si>
+    <t>Total Remaining</t>
+  </si>
+  <si>
+    <t>Total in WIP List [Zotero]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -8632,6 +8798,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
     </font>
   </fonts>
   <fills count="5">
@@ -9008,17 +9179,69 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="J26" dT="2026-07-26T14:17:52.96" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{8FFD76D4-7893-40DB-82DF-8E1BEF512ABF}">
+    <text>It’s Quantum-Inspired through math, not an actual QCNN</text>
+  </threadedComment>
+  <threadedComment ref="J44" dT="2026-07-26T14:17:31.54" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{A4251980-DD93-4931-A79F-2208C274FC20}">
+    <text>Retracted Paper</text>
+  </threadedComment>
+  <threadedComment ref="J45" dT="2026-07-26T17:08:04.13" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{FD33AB07-11EB-4417-BC00-9F6717F8363D}">
+    <text>MNIST Dataset, potential man paper</text>
+  </threadedComment>
   <threadedComment ref="H61" dT="2026-07-14T21:23:09.31" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{A8621180-8332-4067-A5C3-427EEEAA550B}">
     <text>If not EC4, then EC9</text>
   </threadedComment>
   <threadedComment ref="H129" dT="2026-07-16T05:20:42.92" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{5FCB09E3-43CE-4F41-B07E-5555D6847BA9}">
     <text>Would also be EC9</text>
   </threadedComment>
+  <threadedComment ref="J134" dT="2026-07-26T14:17:25.09" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{4C18BE0C-B936-4C12-970B-A1C978A3A429}">
+    <text>Retracted Paper</text>
+  </threadedComment>
   <threadedComment ref="H142" dT="2026-07-16T05:21:04.61" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{742400F8-FC12-463E-BF7C-44472F707647}">
     <text>EC9 aswell</text>
   </threadedComment>
+  <threadedComment ref="J188" dT="2026-07-26T14:16:55.47" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{AECB7639-3D48-44A5-A023-E6D739E33DBC}">
+    <text>Mandarin Language</text>
+  </threadedComment>
+  <threadedComment ref="J248" dT="2026-07-26T14:16:45.08" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{49984621-F60C-4B95-B404-A070273AAB9E}">
+    <text>MNIST Dataset</text>
+  </threadedComment>
+  <threadedComment ref="J291" dT="2026-07-26T17:20:58.57" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{D4CD819D-9741-4F3F-B1F1-A9EDE1B95C3D}">
+    <text>MNIST Dataset, author acknowledges it</text>
+  </threadedComment>
   <threadedComment ref="H338" dT="2026-07-14T21:59:11.48" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{3BCE51DA-E03A-42CE-BCF4-42F3B17B3F4F}">
     <text>Would’ve loved to use this paper :(</text>
+  </threadedComment>
+  <threadedComment ref="J378" dT="2026-07-26T16:15:24.50" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{6C607B97-DBE1-4B9B-912B-FC5F378C78F8}">
+    <text>Tough Case, needs review:
+- Pros:
+Implementation of a QCNN
+- Cons:
+Benchmarking purpose</text>
+  </threadedComment>
+  <threadedComment ref="J380" dT="2026-07-26T14:16:17.18" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{9B71B6F6-1440-45C7-B9C6-3D3353E0127E}">
+    <text>No QCNN Application</text>
+  </threadedComment>
+  <threadedComment ref="J404" dT="2026-07-26T16:34:55.10" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{9A96E512-3F53-4A8F-86C6-E13A0AA03D5D}">
+    <text>Shouldn’t have been included in stage 1, didn’t know what the Iris dataset was about-</text>
+  </threadedComment>
+  <threadedComment ref="J489" dT="2026-07-26T16:44:14.20" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{74FC4EA6-7D43-442D-AC4B-3B99C2479B6D}">
+    <text>MNIST &amp; FMNIST Dataset</text>
+  </threadedComment>
+  <threadedComment ref="J502" dT="2026-07-26T14:16:00.57" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{31E0DE7F-8E71-41E9-98C2-32C7133F7B0E}">
+    <text>Review</text>
+  </threadedComment>
+  <threadedComment ref="J513" dT="2026-07-26T17:46:02.05" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{332BDD9A-D5F7-4A8F-BA56-7686D80374CB}">
+    <text>MNIST, Autonomous Driving is theoretical and not an application</text>
+  </threadedComment>
+  <threadedComment ref="J521" dT="2026-07-25T20:30:53.20" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{F0C16F01-077A-4435-AC9D-36801D87E965}">
+    <text>MNIST Dataset</text>
+  </threadedComment>
+  <threadedComment ref="J528" dT="2026-07-26T16:54:15.01" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{890B958C-615A-4B5C-8D18-10B0C1B52873}">
+    <text>Good Proposal, only applied against MNIST &amp; FMNIST :(</text>
+  </threadedComment>
+  <threadedComment ref="J547" dT="2026-07-26T17:05:54.41" personId="{8B8B8FFE-33D8-4E42-AD02-3B073D1E92A1}" id="{C58A61C8-AE69-4687-8BF9-249CAA893C01}">
+    <text>Could be interpreted as theoretical, but case studies are relevant and applicable(?)</text>
   </threadedComment>
 </ThreadedComments>
 </file>
@@ -9048,7 +9271,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="44" customWidth="1"/>
@@ -9242,7 +9465,7 @@
       </c>
       <c r="B27">
         <f>COUNTA(Screening!I2:I548)</f>
-        <v>55</v>
+        <v>76</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -9251,7 +9474,7 @@
       </c>
       <c r="B28">
         <f>COUNTIF(Screening!I2:I548,"Exclude")</f>
-        <v>55</v>
+        <v>69</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -9260,82 +9483,100 @@
       </c>
       <c r="B29" s="3">
         <f>COUNTIF(Screening!I2:I548,"Include")</f>
-        <v>0</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>2842</v>
+      </c>
+      <c r="B30" s="3">
+        <f>B13-B27</f>
+        <v>194</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
+      <c r="A31" t="s">
+        <v>2843</v>
+      </c>
+      <c r="B31" s="3">
+        <f>B30+B29</f>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>15</v>
       </c>
-      <c r="B32">
+      <c r="B34">
         <f>COUNTIFS(Screening!I2:I548,"Exclude",Screening!J2:J548,"EC1")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>16</v>
       </c>
-      <c r="B33">
+      <c r="B35">
         <f>COUNTIFS(Screening!I2:I548,"Exclude",Screening!J2:J548,"EC2")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>17</v>
-      </c>
-      <c r="B34">
-        <f>COUNTIFS(Screening!I2:I548,"Exclude",Screening!J2:J548,"EC3")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>18</v>
-      </c>
-      <c r="B35">
-        <f>COUNTIFS(Screening!I2:I548,"Exclude",Screening!J2:J548,"EC4")</f>
-        <v>0</v>
-      </c>
-    </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>17</v>
+      </c>
+      <c r="B36">
+        <f>COUNTIFS(Screening!I2:I548,"Exclude",Screening!J2:J548,"EC3")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>18</v>
+      </c>
+      <c r="B37">
+        <f>COUNTIFS(Screening!I2:I548,"Exclude",Screening!J2:J548,"EC4")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>19</v>
       </c>
-      <c r="B36">
+      <c r="B38">
         <f>COUNTIFS(Screening!I2:I548,"Exclude",Screening!J2:J548,"EC5")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>20</v>
       </c>
-      <c r="B37">
+      <c r="B39">
         <f>COUNTIFS(Screening!I2:I548,"Exclude",Screening!J2:J548,"EC6")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>2708</v>
       </c>
-      <c r="B38">
+      <c r="B40">
         <f>COUNTIFS(Screening!I3:I549,"Exclude",Screening!J3:J549,"EC7")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>2837</v>
       </c>
-      <c r="B39">
+      <c r="B41">
         <f>COUNTIFS(Screening!I4:I550,"Exclude",Screening!J4:J550,"EC8")</f>
         <v>54</v>
       </c>
@@ -9548,7 +9789,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>318</v>
       </c>
@@ -9586,7 +9827,7 @@
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
     </row>
-    <row r="7" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="120" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>13</v>
       </c>
@@ -9607,8 +9848,12 @@
       <c r="H7" s="6" t="s">
         <v>2646</v>
       </c>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
+      <c r="I7" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>2838</v>
+      </c>
       <c r="K7" s="5" t="s">
         <v>110</v>
       </c>
@@ -9786,7 +10031,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" ht="180" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>482</v>
       </c>
@@ -9811,8 +10056,12 @@
       <c r="H13" s="6" t="s">
         <v>2678</v>
       </c>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
+      <c r="I13" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>56</v>
+      </c>
       <c r="K13" s="5" t="s">
         <v>2283</v>
       </c>
@@ -9820,7 +10069,7 @@
       <c r="M13" s="5"/>
       <c r="N13" s="5"/>
     </row>
-    <row r="14" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" ht="150" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>460</v>
       </c>
@@ -9845,8 +10094,12 @@
       <c r="H14" s="6" t="s">
         <v>2690</v>
       </c>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
+      <c r="I14" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>2838</v>
+      </c>
       <c r="K14" s="5" t="s">
         <v>2185</v>
       </c>
@@ -9854,7 +10107,7 @@
       <c r="M14" s="5"/>
       <c r="N14" s="5"/>
     </row>
-    <row r="15" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>408</v>
       </c>
@@ -9892,7 +10145,7 @@
       <c r="M15" s="5"/>
       <c r="N15" s="5"/>
     </row>
-    <row r="16" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" ht="225" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
         <v>87</v>
       </c>
@@ -9917,8 +10170,12 @@
       <c r="H16" s="6" t="s">
         <v>2589</v>
       </c>
-      <c r="I16" s="6"/>
-      <c r="J16" s="6"/>
+      <c r="I16" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>2838</v>
+      </c>
       <c r="K16" s="5" t="s">
         <v>459</v>
       </c>
@@ -9926,7 +10183,7 @@
       <c r="M16" s="5"/>
       <c r="N16" s="5"/>
     </row>
-    <row r="17" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="180" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
         <v>31</v>
       </c>
@@ -9947,8 +10204,12 @@
       <c r="H17" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="I17" s="6"/>
-      <c r="J17" s="6"/>
+      <c r="I17" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>2838</v>
+      </c>
       <c r="K17" s="5" t="s">
         <v>205</v>
       </c>
@@ -10098,7 +10359,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="240" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" ht="240" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
         <v>118</v>
       </c>
@@ -10236,7 +10497,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="300" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" ht="165" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
         <v>382</v>
       </c>
@@ -10259,8 +10520,12 @@
       <c r="H26" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="I26" s="6"/>
-      <c r="J26" s="6"/>
+      <c r="I26" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J26" s="6" t="s">
+        <v>56</v>
+      </c>
       <c r="K26" s="5" t="s">
         <v>1837</v>
       </c>
@@ -10402,7 +10667,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" ht="255" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
         <v>330</v>
       </c>
@@ -10440,7 +10705,7 @@
       <c r="M31" s="5"/>
       <c r="N31" s="5"/>
     </row>
-    <row r="32" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
         <v>268</v>
       </c>
@@ -10510,7 +10775,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
         <v>475</v>
       </c>
@@ -10544,7 +10809,7 @@
       <c r="M34" s="5"/>
       <c r="N34" s="5"/>
     </row>
-    <row r="35" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
         <v>449</v>
       </c>
@@ -10770,7 +11035,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="42" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" ht="270" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="5">
         <v>176</v>
       </c>
@@ -10804,7 +11069,7 @@
       <c r="M42" s="5"/>
       <c r="N42" s="5"/>
     </row>
-    <row r="43" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="5">
         <v>539</v>
       </c>
@@ -10838,7 +11103,7 @@
       <c r="M43" s="5"/>
       <c r="N43" s="5"/>
     </row>
-    <row r="44" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" ht="255" x14ac:dyDescent="0.25">
       <c r="A44" s="5">
         <v>215</v>
       </c>
@@ -10876,7 +11141,7 @@
       <c r="M44" s="5"/>
       <c r="N44" s="5"/>
     </row>
-    <row r="45" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" ht="120" x14ac:dyDescent="0.25">
       <c r="A45" s="5">
         <v>16</v>
       </c>
@@ -10899,8 +11164,12 @@
       <c r="H45" s="6" t="s">
         <v>2648</v>
       </c>
-      <c r="I45" s="6"/>
-      <c r="J45" s="6"/>
+      <c r="I45" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J45" s="6" t="s">
+        <v>2642</v>
+      </c>
       <c r="K45" s="5" t="s">
         <v>125</v>
       </c>
@@ -10942,7 +11211,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" ht="315" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="5">
         <v>404</v>
       </c>
@@ -10980,7 +11249,7 @@
       <c r="M47" s="5"/>
       <c r="N47" s="5"/>
     </row>
-    <row r="48" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" ht="240" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="5">
         <v>61</v>
       </c>
@@ -11044,7 +11313,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="50" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="5">
         <v>44</v>
       </c>
@@ -11172,7 +11441,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="54" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" ht="225" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="5">
         <v>407</v>
       </c>
@@ -11206,7 +11475,7 @@
       <c r="M54" s="5"/>
       <c r="N54" s="5"/>
     </row>
-    <row r="55" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" ht="240" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="5">
         <v>278</v>
       </c>
@@ -11240,7 +11509,7 @@
       <c r="M55" s="5"/>
       <c r="N55" s="5"/>
     </row>
-    <row r="56" spans="1:14" ht="105" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="5">
         <v>195</v>
       </c>
@@ -11278,7 +11547,7 @@
       <c r="M56" s="5"/>
       <c r="N56" s="5"/>
     </row>
-    <row r="57" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="5">
         <v>130</v>
       </c>
@@ -11348,7 +11617,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="59" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="5">
         <v>54</v>
       </c>
@@ -11444,7 +11713,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="62" spans="1:14" ht="240" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5">
         <v>92</v>
       </c>
@@ -11648,7 +11917,7 @@
       <c r="M67" s="5"/>
       <c r="N67" s="5"/>
     </row>
-    <row r="68" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="5">
         <v>108</v>
       </c>
@@ -11720,7 +11989,7 @@
       <c r="M69" s="5"/>
       <c r="N69" s="5"/>
     </row>
-    <row r="70" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="5">
         <v>454</v>
       </c>
@@ -11928,7 +12197,7 @@
       <c r="M75" s="5"/>
       <c r="N75" s="5"/>
     </row>
-    <row r="76" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="5">
         <v>240</v>
       </c>
@@ -11962,7 +12231,7 @@
       <c r="M76" s="5"/>
       <c r="N76" s="5"/>
     </row>
-    <row r="77" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="5">
         <v>520</v>
       </c>
@@ -12064,7 +12333,7 @@
       <c r="M79" s="5"/>
       <c r="N79" s="5"/>
     </row>
-    <row r="80" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:14" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="5">
         <v>306</v>
       </c>
@@ -12166,7 +12435,7 @@
       <c r="M82" s="5"/>
       <c r="N82" s="5"/>
     </row>
-    <row r="83" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="5">
         <v>248</v>
       </c>
@@ -12200,7 +12469,7 @@
       <c r="M83" s="5"/>
       <c r="N83" s="5"/>
     </row>
-    <row r="84" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="5">
         <v>377</v>
       </c>
@@ -12302,7 +12571,7 @@
       <c r="M86" s="5"/>
       <c r="N86" s="5"/>
     </row>
-    <row r="87" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:14" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="5">
         <v>177</v>
       </c>
@@ -12336,7 +12605,7 @@
       <c r="M87" s="5"/>
       <c r="N87" s="5"/>
     </row>
-    <row r="88" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:14" ht="240" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="5">
         <v>140</v>
       </c>
@@ -12404,7 +12673,7 @@
       <c r="M89" s="5"/>
       <c r="N89" s="5"/>
     </row>
-    <row r="90" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="5">
         <v>196</v>
       </c>
@@ -12438,7 +12707,7 @@
       <c r="M90" s="5"/>
       <c r="N90" s="5"/>
     </row>
-    <row r="91" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="5">
         <v>41</v>
       </c>
@@ -12470,7 +12739,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="92" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="5">
         <v>358</v>
       </c>
@@ -12504,7 +12773,7 @@
       <c r="M92" s="5"/>
       <c r="N92" s="5"/>
     </row>
-    <row r="93" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="5">
         <v>412</v>
       </c>
@@ -12542,7 +12811,7 @@
       <c r="M93" s="5"/>
       <c r="N93" s="5"/>
     </row>
-    <row r="94" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:14" ht="360" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="5">
         <v>320</v>
       </c>
@@ -12576,7 +12845,7 @@
       <c r="M94" s="5"/>
       <c r="N94" s="5"/>
     </row>
-    <row r="95" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="5">
         <v>531</v>
       </c>
@@ -12614,7 +12883,7 @@
       <c r="M95" s="5"/>
       <c r="N95" s="5"/>
     </row>
-    <row r="96" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="5">
         <v>457</v>
       </c>
@@ -12648,7 +12917,7 @@
       <c r="M96" s="5"/>
       <c r="N96" s="5"/>
     </row>
-    <row r="97" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="5">
         <v>357</v>
       </c>
@@ -12750,7 +13019,7 @@
       <c r="M99" s="5"/>
       <c r="N99" s="5"/>
     </row>
-    <row r="100" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:14" ht="225" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="5">
         <v>131</v>
       </c>
@@ -12852,7 +13121,7 @@
       <c r="M102" s="5"/>
       <c r="N102" s="5"/>
     </row>
-    <row r="103" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="5">
         <v>280</v>
       </c>
@@ -12924,7 +13193,7 @@
       <c r="M104" s="5"/>
       <c r="N104" s="5"/>
     </row>
-    <row r="105" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:14" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="5">
         <v>252</v>
       </c>
@@ -13026,7 +13295,7 @@
       <c r="M107" s="5"/>
       <c r="N107" s="5"/>
     </row>
-    <row r="108" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="5">
         <v>463</v>
       </c>
@@ -13064,7 +13333,7 @@
       <c r="M108" s="5"/>
       <c r="N108" s="5"/>
     </row>
-    <row r="109" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="5">
         <v>263</v>
       </c>
@@ -13132,7 +13401,7 @@
       <c r="M110" s="5"/>
       <c r="N110" s="5"/>
     </row>
-    <row r="111" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="5">
         <v>349</v>
       </c>
@@ -13166,7 +13435,7 @@
       <c r="M111" s="5"/>
       <c r="N111" s="5"/>
     </row>
-    <row r="112" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:14" ht="225" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" s="5">
         <v>33</v>
       </c>
@@ -13198,7 +13467,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="113" spans="1:14" ht="285" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" s="5">
         <v>286</v>
       </c>
@@ -13236,7 +13505,7 @@
       <c r="M113" s="5"/>
       <c r="N113" s="5"/>
     </row>
-    <row r="114" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:14" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" s="5">
         <v>290</v>
       </c>
@@ -13274,7 +13543,7 @@
       <c r="M114" s="5"/>
       <c r="N114" s="5"/>
     </row>
-    <row r="115" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" s="5">
         <v>133</v>
       </c>
@@ -13376,7 +13645,7 @@
       <c r="M117" s="5"/>
       <c r="N117" s="5"/>
     </row>
-    <row r="118" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="5">
         <v>527</v>
       </c>
@@ -13410,7 +13679,7 @@
       <c r="M118" s="5"/>
       <c r="N118" s="5"/>
     </row>
-    <row r="119" spans="1:14" ht="240" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" s="5">
         <v>401</v>
       </c>
@@ -13444,7 +13713,7 @@
       <c r="M119" s="5"/>
       <c r="N119" s="5"/>
     </row>
-    <row r="120" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:14" ht="330" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" s="5">
         <v>368</v>
       </c>
@@ -13516,7 +13785,7 @@
       <c r="M121" s="5"/>
       <c r="N121" s="5"/>
     </row>
-    <row r="122" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:14" ht="270" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" s="5">
         <v>254</v>
       </c>
@@ -13584,7 +13853,7 @@
       <c r="M123" s="5"/>
       <c r="N123" s="5"/>
     </row>
-    <row r="124" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:14" ht="285" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" s="5">
         <v>264</v>
       </c>
@@ -13618,7 +13887,7 @@
       <c r="M124" s="5"/>
       <c r="N124" s="5"/>
     </row>
-    <row r="125" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" s="5">
         <v>228</v>
       </c>
@@ -13652,7 +13921,7 @@
       <c r="M125" s="5"/>
       <c r="N125" s="5"/>
     </row>
-    <row r="126" spans="1:14" ht="240" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:14" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" s="5">
         <v>394</v>
       </c>
@@ -13690,7 +13959,7 @@
       <c r="M126" s="5"/>
       <c r="N126" s="5"/>
     </row>
-    <row r="127" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:14" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" s="5">
         <v>235</v>
       </c>
@@ -13792,7 +14061,7 @@
       <c r="M129" s="5"/>
       <c r="N129" s="5"/>
     </row>
-    <row r="130" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" s="5">
         <v>321</v>
       </c>
@@ -13826,7 +14095,7 @@
       <c r="M130" s="5"/>
       <c r="N130" s="5"/>
     </row>
-    <row r="131" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" s="5">
         <v>545</v>
       </c>
@@ -13860,7 +14129,7 @@
       <c r="M131" s="5"/>
       <c r="N131" s="5"/>
     </row>
-    <row r="132" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" s="5">
         <v>519</v>
       </c>
@@ -13928,7 +14197,7 @@
       <c r="M133" s="5"/>
       <c r="N133" s="5"/>
     </row>
-    <row r="134" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:14" ht="150" x14ac:dyDescent="0.25">
       <c r="A134" s="5">
         <v>523</v>
       </c>
@@ -13953,8 +14222,12 @@
       <c r="H134" s="6" t="s">
         <v>2659</v>
       </c>
-      <c r="I134" s="6"/>
-      <c r="J134" s="6"/>
+      <c r="I134" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J134" s="6" t="s">
+        <v>2578</v>
+      </c>
       <c r="K134" s="5" t="s">
         <v>2462</v>
       </c>
@@ -14030,7 +14303,7 @@
       <c r="M136" s="5"/>
       <c r="N136" s="5"/>
     </row>
-    <row r="137" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:14" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" s="5">
         <v>82</v>
       </c>
@@ -14064,7 +14337,7 @@
       <c r="M137" s="5"/>
       <c r="N137" s="5"/>
     </row>
-    <row r="138" spans="1:14" ht="285" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" s="5">
         <v>102</v>
       </c>
@@ -14098,7 +14371,7 @@
       <c r="M138" s="5"/>
       <c r="N138" s="5"/>
     </row>
-    <row r="139" spans="1:14" ht="270" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:14" ht="225" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" s="5">
         <v>181</v>
       </c>
@@ -14170,7 +14443,7 @@
       <c r="M140" s="5"/>
       <c r="N140" s="5"/>
     </row>
-    <row r="141" spans="1:14" ht="240" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" s="5">
         <v>67</v>
       </c>
@@ -14238,7 +14511,7 @@
       <c r="M142" s="5"/>
       <c r="N142" s="5"/>
     </row>
-    <row r="143" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:14" ht="255" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" s="5">
         <v>438</v>
       </c>
@@ -14442,7 +14715,7 @@
       <c r="M148" s="5"/>
       <c r="N148" s="5"/>
     </row>
-    <row r="149" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:14" ht="240" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" s="5">
         <v>21</v>
       </c>
@@ -14610,7 +14883,7 @@
       <c r="M153" s="5"/>
       <c r="N153" s="5"/>
     </row>
-    <row r="154" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="5">
         <v>430</v>
       </c>
@@ -14678,7 +14951,7 @@
       <c r="M155" s="5"/>
       <c r="N155" s="5"/>
     </row>
-    <row r="156" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" s="5">
         <v>124</v>
       </c>
@@ -14712,7 +14985,7 @@
       <c r="M156" s="5"/>
       <c r="N156" s="5"/>
     </row>
-    <row r="157" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:14" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="5">
         <v>91</v>
       </c>
@@ -14848,7 +15121,7 @@
       <c r="M160" s="5"/>
       <c r="N160" s="5"/>
     </row>
-    <row r="161" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" s="5">
         <v>256</v>
       </c>
@@ -14916,7 +15189,7 @@
       <c r="M162" s="5"/>
       <c r="N162" s="5"/>
     </row>
-    <row r="163" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" s="5">
         <v>53</v>
       </c>
@@ -15016,7 +15289,7 @@
       <c r="M165" s="5"/>
       <c r="N165" s="5"/>
     </row>
-    <row r="166" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" s="5">
         <v>136</v>
       </c>
@@ -15050,7 +15323,7 @@
       <c r="M166" s="5"/>
       <c r="N166" s="5"/>
     </row>
-    <row r="167" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" s="5">
         <v>119</v>
       </c>
@@ -15084,7 +15357,7 @@
       <c r="M167" s="5"/>
       <c r="N167" s="5"/>
     </row>
-    <row r="168" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168" s="5">
         <v>483</v>
       </c>
@@ -15156,7 +15429,7 @@
       <c r="M169" s="5"/>
       <c r="N169" s="5"/>
     </row>
-    <row r="170" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170" s="5">
         <v>266</v>
       </c>
@@ -15224,7 +15497,7 @@
       <c r="M171" s="5"/>
       <c r="N171" s="5"/>
     </row>
-    <row r="172" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:14" ht="270" x14ac:dyDescent="0.25">
       <c r="A172" s="5">
         <v>476</v>
       </c>
@@ -15249,8 +15522,12 @@
       <c r="H172" s="6" t="s">
         <v>2631</v>
       </c>
-      <c r="I172" s="6"/>
-      <c r="J172" s="6"/>
+      <c r="I172" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J172" s="6" t="s">
+        <v>2838</v>
+      </c>
       <c r="K172" s="5" t="s">
         <v>2256</v>
       </c>
@@ -15392,7 +15669,7 @@
       <c r="M176" s="5"/>
       <c r="N176" s="5"/>
     </row>
-    <row r="177" spans="1:14" ht="270" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177" s="5">
         <v>487</v>
       </c>
@@ -15426,7 +15703,7 @@
       <c r="M177" s="5"/>
       <c r="N177" s="5"/>
     </row>
-    <row r="178" spans="1:14" ht="105" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178" s="5">
         <v>79</v>
       </c>
@@ -15562,7 +15839,7 @@
       <c r="M181" s="5"/>
       <c r="N181" s="5"/>
     </row>
-    <row r="182" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182" s="5">
         <v>443</v>
       </c>
@@ -15596,7 +15873,7 @@
       <c r="M182" s="5"/>
       <c r="N182" s="5"/>
     </row>
-    <row r="183" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" s="5">
         <v>294</v>
       </c>
@@ -15630,7 +15907,7 @@
       <c r="M183" s="5"/>
       <c r="N183" s="5"/>
     </row>
-    <row r="184" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:14" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A184" s="5">
         <v>302</v>
       </c>
@@ -15702,7 +15979,7 @@
       <c r="M185" s="5"/>
       <c r="N185" s="5"/>
     </row>
-    <row r="186" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186" s="5">
         <v>94</v>
       </c>
@@ -15770,7 +16047,7 @@
       <c r="M187" s="5"/>
       <c r="N187" s="5"/>
     </row>
-    <row r="188" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:14" ht="165" x14ac:dyDescent="0.25">
       <c r="A188" s="5">
         <v>342</v>
       </c>
@@ -15795,8 +16072,12 @@
       <c r="H188" s="6" t="s">
         <v>2827</v>
       </c>
-      <c r="I188" s="6"/>
-      <c r="J188" s="6"/>
+      <c r="I188" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J188" s="6" t="s">
+        <v>2576</v>
+      </c>
       <c r="K188" s="5" t="s">
         <v>1656</v>
       </c>
@@ -15872,7 +16153,7 @@
       <c r="M190" s="5"/>
       <c r="N190" s="5"/>
     </row>
-    <row r="191" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A191" s="5">
         <v>83</v>
       </c>
@@ -15906,7 +16187,7 @@
       <c r="M191" s="5"/>
       <c r="N191" s="5"/>
     </row>
-    <row r="192" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A192" s="5">
         <v>369</v>
       </c>
@@ -15938,7 +16219,7 @@
       <c r="M192" s="5"/>
       <c r="N192" s="5"/>
     </row>
-    <row r="193" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:14" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A193" s="5">
         <v>187</v>
       </c>
@@ -15972,7 +16253,7 @@
       <c r="M193" s="5"/>
       <c r="N193" s="5"/>
     </row>
-    <row r="194" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A194" s="5">
         <v>447</v>
       </c>
@@ -16040,7 +16321,7 @@
       <c r="M195" s="5"/>
       <c r="N195" s="5"/>
     </row>
-    <row r="196" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:14" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196" s="5">
         <v>198</v>
       </c>
@@ -16074,7 +16355,7 @@
       <c r="M196" s="5"/>
       <c r="N196" s="5"/>
     </row>
-    <row r="197" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197" s="5">
         <v>328</v>
       </c>
@@ -16142,7 +16423,7 @@
       <c r="M198" s="5"/>
       <c r="N198" s="5"/>
     </row>
-    <row r="199" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:14" ht="270" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199" s="5">
         <v>509</v>
       </c>
@@ -16346,7 +16627,7 @@
       <c r="M204" s="5"/>
       <c r="N204" s="5"/>
     </row>
-    <row r="205" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A205" s="5">
         <v>299</v>
       </c>
@@ -16414,7 +16695,7 @@
       <c r="M206" s="5"/>
       <c r="N206" s="5"/>
     </row>
-    <row r="207" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:14" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207" s="5">
         <v>456</v>
       </c>
@@ -16448,7 +16729,7 @@
       <c r="M207" s="5"/>
       <c r="N207" s="5"/>
     </row>
-    <row r="208" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A208" s="5">
         <v>5</v>
       </c>
@@ -16484,7 +16765,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="209" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A209" s="5">
         <v>153</v>
       </c>
@@ -16552,7 +16833,7 @@
       <c r="M210" s="5"/>
       <c r="N210" s="5"/>
     </row>
-    <row r="211" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A211" s="5">
         <v>239</v>
       </c>
@@ -16658,7 +16939,7 @@
       <c r="M213" s="5"/>
       <c r="N213" s="5"/>
     </row>
-    <row r="214" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:14" ht="225" hidden="1" x14ac:dyDescent="0.25">
       <c r="A214" s="5">
         <v>535</v>
       </c>
@@ -16692,7 +16973,7 @@
       <c r="M214" s="5"/>
       <c r="N214" s="5"/>
     </row>
-    <row r="215" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A215" s="5">
         <v>537</v>
       </c>
@@ -16730,7 +17011,7 @@
       <c r="M215" s="5"/>
       <c r="N215" s="5"/>
     </row>
-    <row r="216" spans="1:14" ht="255" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:14" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A216" s="5">
         <v>425</v>
       </c>
@@ -16904,7 +17185,7 @@
       <c r="M220" s="5"/>
       <c r="N220" s="5"/>
     </row>
-    <row r="221" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A221" s="5">
         <v>435</v>
       </c>
@@ -17004,7 +17285,7 @@
       <c r="M223" s="5"/>
       <c r="N223" s="5"/>
     </row>
-    <row r="224" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A224" s="5">
         <v>142</v>
       </c>
@@ -17038,7 +17319,7 @@
       <c r="M224" s="5"/>
       <c r="N224" s="5"/>
     </row>
-    <row r="225" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:14" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A225" s="5">
         <v>213</v>
       </c>
@@ -17106,7 +17387,7 @@
       <c r="M226" s="5"/>
       <c r="N226" s="5"/>
     </row>
-    <row r="227" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A227" s="5">
         <v>477</v>
       </c>
@@ -17174,7 +17455,7 @@
       <c r="M228" s="5"/>
       <c r="N228" s="5"/>
     </row>
-    <row r="229" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:14" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A229" s="5">
         <v>246</v>
       </c>
@@ -17208,7 +17489,7 @@
       <c r="M229" s="5"/>
       <c r="N229" s="5"/>
     </row>
-    <row r="230" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:14" ht="255" hidden="1" x14ac:dyDescent="0.25">
       <c r="A230" s="5">
         <v>260</v>
       </c>
@@ -17242,7 +17523,7 @@
       <c r="M230" s="5"/>
       <c r="N230" s="5"/>
     </row>
-    <row r="231" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A231" s="5">
         <v>193</v>
       </c>
@@ -17276,7 +17557,7 @@
       <c r="M231" s="5"/>
       <c r="N231" s="5"/>
     </row>
-    <row r="232" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A232" s="5">
         <v>511</v>
       </c>
@@ -17378,7 +17659,7 @@
       <c r="M234" s="5"/>
       <c r="N234" s="5"/>
     </row>
-    <row r="235" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A235" s="5">
         <v>166</v>
       </c>
@@ -17412,7 +17693,7 @@
       <c r="M235" s="5"/>
       <c r="N235" s="5"/>
     </row>
-    <row r="236" spans="1:14" ht="105" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A236" s="5">
         <v>214</v>
       </c>
@@ -17480,7 +17761,7 @@
       <c r="M237" s="5"/>
       <c r="N237" s="5"/>
     </row>
-    <row r="238" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:14" ht="240" hidden="1" x14ac:dyDescent="0.25">
       <c r="A238" s="5">
         <v>387</v>
       </c>
@@ -17548,7 +17829,7 @@
       <c r="M239" s="5"/>
       <c r="N239" s="5"/>
     </row>
-    <row r="240" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A240" s="5">
         <v>121</v>
       </c>
@@ -17582,7 +17863,7 @@
       <c r="M240" s="5"/>
       <c r="N240" s="5"/>
     </row>
-    <row r="241" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:14" ht="225" hidden="1" x14ac:dyDescent="0.25">
       <c r="A241" s="5">
         <v>165</v>
       </c>
@@ -17650,7 +17931,7 @@
       <c r="M242" s="5"/>
       <c r="N242" s="5"/>
     </row>
-    <row r="243" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A243" s="5">
         <v>171</v>
       </c>
@@ -17786,7 +18067,7 @@
       <c r="M246" s="5"/>
       <c r="N246" s="5"/>
     </row>
-    <row r="247" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A247" s="5">
         <v>418</v>
       </c>
@@ -17824,7 +18105,7 @@
       <c r="M247" s="5"/>
       <c r="N247" s="5"/>
     </row>
-    <row r="248" spans="1:14" ht="285" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:14" ht="210" x14ac:dyDescent="0.25">
       <c r="A248" s="5">
         <v>43</v>
       </c>
@@ -17845,8 +18126,12 @@
       <c r="H248" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="I248" s="6"/>
-      <c r="J248" s="6"/>
+      <c r="I248" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J248" s="6" t="s">
+        <v>2642</v>
+      </c>
       <c r="K248" s="5" t="s">
         <v>258</v>
       </c>
@@ -17856,7 +18141,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="249" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A249" s="5">
         <v>350</v>
       </c>
@@ -17958,7 +18243,7 @@
       <c r="M251" s="5"/>
       <c r="N251" s="5"/>
     </row>
-    <row r="252" spans="1:14" ht="270" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:14" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A252" s="5">
         <v>160</v>
       </c>
@@ -17996,7 +18281,7 @@
       <c r="M252" s="5"/>
       <c r="N252" s="5"/>
     </row>
-    <row r="253" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A253" s="5">
         <v>190</v>
       </c>
@@ -18064,7 +18349,7 @@
       <c r="M254" s="5"/>
       <c r="N254" s="5"/>
     </row>
-    <row r="255" spans="1:14" ht="270" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A255" s="5">
         <v>279</v>
       </c>
@@ -18132,7 +18417,7 @@
       <c r="M256" s="5"/>
       <c r="N256" s="5"/>
     </row>
-    <row r="257" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A257" s="5">
         <v>305</v>
       </c>
@@ -18268,7 +18553,7 @@
       <c r="M260" s="5"/>
       <c r="N260" s="5"/>
     </row>
-    <row r="261" spans="1:14" ht="255" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A261" s="5">
         <v>47</v>
       </c>
@@ -18368,7 +18653,7 @@
       <c r="M263" s="5"/>
       <c r="N263" s="5"/>
     </row>
-    <row r="264" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A264" s="5">
         <v>155</v>
       </c>
@@ -18402,7 +18687,7 @@
       <c r="M264" s="5"/>
       <c r="N264" s="5"/>
     </row>
-    <row r="265" spans="1:14" ht="285" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A265" s="5">
         <v>90</v>
       </c>
@@ -18470,7 +18755,7 @@
       <c r="M266" s="5"/>
       <c r="N266" s="5"/>
     </row>
-    <row r="267" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A267" s="5">
         <v>544</v>
       </c>
@@ -18508,7 +18793,7 @@
       <c r="M267" s="5"/>
       <c r="N267" s="5"/>
     </row>
-    <row r="268" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A268" s="5">
         <v>466</v>
       </c>
@@ -18546,7 +18831,7 @@
       <c r="M268" s="5"/>
       <c r="N268" s="5"/>
     </row>
-    <row r="269" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A269" s="5">
         <v>423</v>
       </c>
@@ -18784,7 +19069,7 @@
       <c r="M275" s="5"/>
       <c r="N275" s="5"/>
     </row>
-    <row r="276" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A276" s="5">
         <v>405</v>
       </c>
@@ -18886,7 +19171,7 @@
       <c r="M278" s="5"/>
       <c r="N278" s="5"/>
     </row>
-    <row r="279" spans="1:14" ht="240" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A279" s="5">
         <v>117</v>
       </c>
@@ -18924,7 +19209,7 @@
       <c r="M279" s="5"/>
       <c r="N279" s="5"/>
     </row>
-    <row r="280" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A280" s="5">
         <v>234</v>
       </c>
@@ -18958,7 +19243,7 @@
       <c r="M280" s="5"/>
       <c r="N280" s="5"/>
     </row>
-    <row r="281" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A281" s="5">
         <v>395</v>
       </c>
@@ -18992,7 +19277,7 @@
       <c r="M281" s="5"/>
       <c r="N281" s="5"/>
     </row>
-    <row r="282" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:14" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A282" s="5">
         <v>455</v>
       </c>
@@ -19030,7 +19315,7 @@
       <c r="M282" s="5"/>
       <c r="N282" s="5"/>
     </row>
-    <row r="283" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:14" ht="270" hidden="1" x14ac:dyDescent="0.25">
       <c r="A283" s="5">
         <v>251</v>
       </c>
@@ -19064,7 +19349,7 @@
       <c r="M283" s="5"/>
       <c r="N283" s="5"/>
     </row>
-    <row r="284" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:14" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A284" s="5">
         <v>96</v>
       </c>
@@ -19132,7 +19417,7 @@
       <c r="M285" s="5"/>
       <c r="N285" s="5"/>
     </row>
-    <row r="286" spans="1:14" ht="255" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A286" s="5">
         <v>385</v>
       </c>
@@ -19166,7 +19451,7 @@
       <c r="M286" s="5"/>
       <c r="N286" s="5"/>
     </row>
-    <row r="287" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:14" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A287" s="5">
         <v>275</v>
       </c>
@@ -19204,7 +19489,7 @@
       <c r="M287" s="5"/>
       <c r="N287" s="5"/>
     </row>
-    <row r="288" spans="1:14" ht="240" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A288" s="5">
         <v>129</v>
       </c>
@@ -19308,7 +19593,7 @@
       <c r="M290" s="5"/>
       <c r="N290" s="5"/>
     </row>
-    <row r="291" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:14" ht="210" x14ac:dyDescent="0.25">
       <c r="A291" s="5">
         <v>56</v>
       </c>
@@ -19329,8 +19614,12 @@
       <c r="H291" s="6" t="s">
         <v>2581</v>
       </c>
-      <c r="I291" s="6"/>
-      <c r="J291" s="6"/>
+      <c r="I291" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J291" s="6" t="s">
+        <v>2642</v>
+      </c>
       <c r="K291" s="5" t="s">
         <v>312</v>
       </c>
@@ -19374,7 +19663,7 @@
       <c r="M292" s="5"/>
       <c r="N292" s="5"/>
     </row>
-    <row r="293" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A293" s="5">
         <v>399</v>
       </c>
@@ -19408,7 +19697,7 @@
       <c r="M293" s="5"/>
       <c r="N293" s="5"/>
     </row>
-    <row r="294" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:14" ht="225" hidden="1" x14ac:dyDescent="0.25">
       <c r="A294" s="5">
         <v>381</v>
       </c>
@@ -19442,7 +19731,7 @@
       <c r="M294" s="5"/>
       <c r="N294" s="5"/>
     </row>
-    <row r="295" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A295" s="5">
         <v>95</v>
       </c>
@@ -19476,7 +19765,7 @@
       <c r="M295" s="5"/>
       <c r="N295" s="5"/>
     </row>
-    <row r="296" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:14" ht="225" hidden="1" x14ac:dyDescent="0.25">
       <c r="A296" s="5">
         <v>226</v>
       </c>
@@ -19616,7 +19905,7 @@
       <c r="M299" s="5"/>
       <c r="N299" s="5"/>
     </row>
-    <row r="300" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:14" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A300" s="5">
         <v>403</v>
       </c>
@@ -19718,7 +20007,7 @@
       <c r="M302" s="5"/>
       <c r="N302" s="5"/>
     </row>
-    <row r="303" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:14" ht="255" hidden="1" x14ac:dyDescent="0.25">
       <c r="A303" s="5">
         <v>417</v>
       </c>
@@ -19756,7 +20045,7 @@
       <c r="M303" s="5"/>
       <c r="N303" s="5"/>
     </row>
-    <row r="304" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A304" s="5">
         <v>421</v>
       </c>
@@ -19790,7 +20079,7 @@
       <c r="M304" s="5"/>
       <c r="N304" s="5"/>
     </row>
-    <row r="305" spans="1:14" ht="255" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:14" ht="225" hidden="1" x14ac:dyDescent="0.25">
       <c r="A305" s="5">
         <v>503</v>
       </c>
@@ -19824,7 +20113,7 @@
       <c r="M305" s="5"/>
       <c r="N305" s="5"/>
     </row>
-    <row r="306" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A306" s="5">
         <v>490</v>
       </c>
@@ -19858,7 +20147,7 @@
       <c r="M306" s="5"/>
       <c r="N306" s="5"/>
     </row>
-    <row r="307" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A307" s="5">
         <v>329</v>
       </c>
@@ -20198,7 +20487,7 @@
       <c r="M316" s="5"/>
       <c r="N316" s="5"/>
     </row>
-    <row r="317" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A317" s="5">
         <v>365</v>
       </c>
@@ -20266,7 +20555,7 @@
       <c r="M318" s="5"/>
       <c r="N318" s="5"/>
     </row>
-    <row r="319" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A319" s="5">
         <v>379</v>
       </c>
@@ -20334,7 +20623,7 @@
       <c r="M320" s="5"/>
       <c r="N320" s="5"/>
     </row>
-    <row r="321" spans="1:14" ht="360" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A321" s="5">
         <v>347</v>
       </c>
@@ -20368,7 +20657,7 @@
       <c r="M321" s="5"/>
       <c r="N321" s="5"/>
     </row>
-    <row r="322" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:14" ht="270" hidden="1" x14ac:dyDescent="0.25">
       <c r="A322" s="5">
         <v>138</v>
       </c>
@@ -20470,7 +20759,7 @@
       <c r="M324" s="5"/>
       <c r="N324" s="5"/>
     </row>
-    <row r="325" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:14" ht="240" hidden="1" x14ac:dyDescent="0.25">
       <c r="A325" s="5">
         <v>396</v>
       </c>
@@ -20606,7 +20895,7 @@
       <c r="M328" s="5"/>
       <c r="N328" s="5"/>
     </row>
-    <row r="329" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:14" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A329" s="5">
         <v>496</v>
       </c>
@@ -20644,7 +20933,7 @@
       <c r="M329" s="5"/>
       <c r="N329" s="5"/>
     </row>
-    <row r="330" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A330" s="5">
         <v>204</v>
       </c>
@@ -20682,7 +20971,7 @@
       <c r="M330" s="5"/>
       <c r="N330" s="5"/>
     </row>
-    <row r="331" spans="1:14" ht="255" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A331" s="5">
         <v>441</v>
       </c>
@@ -20886,7 +21175,7 @@
       <c r="M336" s="5"/>
       <c r="N336" s="5"/>
     </row>
-    <row r="337" spans="1:14" ht="105" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A337" s="5">
         <v>182</v>
       </c>
@@ -21090,7 +21379,7 @@
       <c r="M342" s="5"/>
       <c r="N342" s="5"/>
     </row>
-    <row r="343" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A343" s="5">
         <v>185</v>
       </c>
@@ -21160,7 +21449,7 @@
       <c r="M344" s="5"/>
       <c r="N344" s="5"/>
     </row>
-    <row r="345" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A345" s="5">
         <v>283</v>
       </c>
@@ -21194,7 +21483,7 @@
       <c r="M345" s="5"/>
       <c r="N345" s="5"/>
     </row>
-    <row r="346" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A346" s="5">
         <v>501</v>
       </c>
@@ -21262,7 +21551,7 @@
       <c r="M347" s="5"/>
       <c r="N347" s="5"/>
     </row>
-    <row r="348" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A348" s="5">
         <v>113</v>
       </c>
@@ -21330,7 +21619,7 @@
       <c r="M349" s="5"/>
       <c r="N349" s="5"/>
     </row>
-    <row r="350" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A350" s="5">
         <v>480</v>
       </c>
@@ -21368,7 +21657,7 @@
       <c r="M350" s="5"/>
       <c r="N350" s="5"/>
     </row>
-    <row r="351" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A351" s="5">
         <v>468</v>
       </c>
@@ -21436,7 +21725,7 @@
       <c r="M352" s="5"/>
       <c r="N352" s="5"/>
     </row>
-    <row r="353" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:14" ht="285" hidden="1" x14ac:dyDescent="0.25">
       <c r="A353" s="5">
         <v>247</v>
       </c>
@@ -21610,7 +21899,7 @@
       <c r="M357" s="5"/>
       <c r="N357" s="5"/>
     </row>
-    <row r="358" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:14" ht="225" hidden="1" x14ac:dyDescent="0.25">
       <c r="A358" s="5">
         <v>224</v>
       </c>
@@ -21648,7 +21937,7 @@
       <c r="M358" s="5"/>
       <c r="N358" s="5"/>
     </row>
-    <row r="359" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:14" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A359" s="5">
         <v>192</v>
       </c>
@@ -21886,7 +22175,7 @@
       <c r="M365" s="5"/>
       <c r="N365" s="5"/>
     </row>
-    <row r="366" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:14" ht="255" hidden="1" x14ac:dyDescent="0.25">
       <c r="A366" s="5">
         <v>304</v>
       </c>
@@ -21988,7 +22277,7 @@
       <c r="M368" s="5"/>
       <c r="N368" s="5"/>
     </row>
-    <row r="369" spans="1:14" ht="330" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A369" s="5">
         <v>437</v>
       </c>
@@ -22022,7 +22311,7 @@
       <c r="M369" s="5"/>
       <c r="N369" s="5"/>
     </row>
-    <row r="370" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A370" s="5">
         <v>293</v>
       </c>
@@ -22124,7 +22413,7 @@
       <c r="M372" s="5"/>
       <c r="N372" s="5"/>
     </row>
-    <row r="373" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A373" s="5">
         <v>546</v>
       </c>
@@ -22192,7 +22481,7 @@
       <c r="M374" s="5"/>
       <c r="N374" s="5"/>
     </row>
-    <row r="375" spans="1:14" ht="105" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A375" s="5">
         <v>230</v>
       </c>
@@ -22260,7 +22549,7 @@
       <c r="M376" s="5"/>
       <c r="N376" s="5"/>
     </row>
-    <row r="377" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:14" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A377" s="5">
         <v>532</v>
       </c>
@@ -22298,7 +22587,7 @@
       <c r="M377" s="5"/>
       <c r="N377" s="5"/>
     </row>
-    <row r="378" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:14" ht="150" x14ac:dyDescent="0.25">
       <c r="A378" s="5">
         <v>34</v>
       </c>
@@ -22319,8 +22608,12 @@
       <c r="H378" s="6" t="s">
         <v>2720</v>
       </c>
-      <c r="I378" s="6"/>
-      <c r="J378" s="6"/>
+      <c r="I378" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="J378" s="6" t="s">
+        <v>2839</v>
+      </c>
       <c r="K378" s="5" t="s">
         <v>219</v>
       </c>
@@ -22364,7 +22657,7 @@
       <c r="M379" s="5"/>
       <c r="N379" s="5"/>
     </row>
-    <row r="380" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:14" ht="225" x14ac:dyDescent="0.25">
       <c r="A380" s="5">
         <v>42</v>
       </c>
@@ -22385,8 +22678,12 @@
       <c r="H380" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="I380" s="6"/>
-      <c r="J380" s="6"/>
+      <c r="I380" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J380" s="6" t="s">
+        <v>56</v>
+      </c>
       <c r="K380" s="5" t="s">
         <v>253</v>
       </c>
@@ -22396,7 +22693,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="381" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:14" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A381" s="5">
         <v>169</v>
       </c>
@@ -22430,7 +22727,7 @@
       <c r="M381" s="5"/>
       <c r="N381" s="5"/>
     </row>
-    <row r="382" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:14" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A382" s="5">
         <v>267</v>
       </c>
@@ -22464,7 +22761,7 @@
       <c r="M382" s="5"/>
       <c r="N382" s="5"/>
     </row>
-    <row r="383" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A383" s="5">
         <v>461</v>
       </c>
@@ -22566,7 +22863,7 @@
       <c r="M385" s="5"/>
       <c r="N385" s="5"/>
     </row>
-    <row r="386" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A386" s="5">
         <v>431</v>
       </c>
@@ -22636,7 +22933,7 @@
       <c r="M387" s="5"/>
       <c r="N387" s="5"/>
     </row>
-    <row r="388" spans="1:14" ht="240" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:14" ht="225" hidden="1" x14ac:dyDescent="0.25">
       <c r="A388" s="5">
         <v>282</v>
       </c>
@@ -22840,7 +23137,7 @@
       <c r="M393" s="5"/>
       <c r="N393" s="5"/>
     </row>
-    <row r="394" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:14" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A394" s="5">
         <v>374</v>
       </c>
@@ -22874,7 +23171,7 @@
       <c r="M394" s="5"/>
       <c r="N394" s="5"/>
     </row>
-    <row r="395" spans="1:14" ht="105" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A395" s="5">
         <v>107</v>
       </c>
@@ -22908,7 +23205,7 @@
       <c r="M395" s="5"/>
       <c r="N395" s="5"/>
     </row>
-    <row r="396" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A396" s="5">
         <v>210</v>
       </c>
@@ -22942,7 +23239,7 @@
       <c r="M396" s="5"/>
       <c r="N396" s="5"/>
     </row>
-    <row r="397" spans="1:14" ht="240" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:14" ht="240" hidden="1" x14ac:dyDescent="0.25">
       <c r="A397" s="5">
         <v>125</v>
       </c>
@@ -23044,7 +23341,7 @@
       <c r="M399" s="5"/>
       <c r="N399" s="5"/>
     </row>
-    <row r="400" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A400" s="5">
         <v>167</v>
       </c>
@@ -23078,7 +23375,7 @@
       <c r="M400" s="5"/>
       <c r="N400" s="5"/>
     </row>
-    <row r="401" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:14" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A401" s="5">
         <v>429</v>
       </c>
@@ -23116,7 +23413,7 @@
       <c r="M401" s="5"/>
       <c r="N401" s="5"/>
     </row>
-    <row r="402" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A402" s="5">
         <v>93</v>
       </c>
@@ -23150,7 +23447,7 @@
       <c r="M402" s="5"/>
       <c r="N402" s="5"/>
     </row>
-    <row r="403" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A403" s="5">
         <v>533</v>
       </c>
@@ -23184,7 +23481,7 @@
       <c r="M403" s="5"/>
       <c r="N403" s="5"/>
     </row>
-    <row r="404" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:14" ht="135" x14ac:dyDescent="0.25">
       <c r="A404" s="5">
         <v>30</v>
       </c>
@@ -23207,8 +23504,12 @@
       <c r="H404" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="I404" s="6"/>
-      <c r="J404" s="6"/>
+      <c r="I404" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J404" s="6" t="s">
+        <v>2642</v>
+      </c>
       <c r="K404" s="5" t="s">
         <v>200</v>
       </c>
@@ -23218,7 +23519,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="405" spans="1:14" ht="315" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:14" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A405" s="5">
         <v>479</v>
       </c>
@@ -23252,7 +23553,7 @@
       <c r="M405" s="5"/>
       <c r="N405" s="5"/>
     </row>
-    <row r="406" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A406" s="5">
         <v>206</v>
       </c>
@@ -23320,7 +23621,7 @@
       <c r="M407" s="5"/>
       <c r="N407" s="5"/>
     </row>
-    <row r="408" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A408" s="5">
         <v>162</v>
       </c>
@@ -23354,7 +23655,7 @@
       <c r="M408" s="5"/>
       <c r="N408" s="5"/>
     </row>
-    <row r="409" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A409" s="5">
         <v>497</v>
       </c>
@@ -23490,7 +23791,7 @@
       <c r="M412" s="5"/>
       <c r="N412" s="5"/>
     </row>
-    <row r="413" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A413" s="5">
         <v>472</v>
       </c>
@@ -23660,7 +23961,7 @@
       <c r="M417" s="5"/>
       <c r="N417" s="5"/>
     </row>
-    <row r="418" spans="1:14" ht="255" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A418" s="5">
         <v>344</v>
       </c>
@@ -23694,7 +23995,7 @@
       <c r="M418" s="5"/>
       <c r="N418" s="5"/>
     </row>
-    <row r="419" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="419" spans="1:14" ht="300" hidden="1" x14ac:dyDescent="0.25">
       <c r="A419" s="5">
         <v>25</v>
       </c>
@@ -23794,7 +24095,7 @@
       <c r="M421" s="5"/>
       <c r="N421" s="5"/>
     </row>
-    <row r="422" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="422" spans="1:14" ht="225" hidden="1" x14ac:dyDescent="0.25">
       <c r="A422" s="5">
         <v>99</v>
       </c>
@@ -23862,7 +24163,7 @@
       <c r="M423" s="5"/>
       <c r="N423" s="5"/>
     </row>
-    <row r="424" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="424" spans="1:14" ht="330" hidden="1" x14ac:dyDescent="0.25">
       <c r="A424" s="5">
         <v>473</v>
       </c>
@@ -23930,7 +24231,7 @@
       <c r="M425" s="5"/>
       <c r="N425" s="5"/>
     </row>
-    <row r="426" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="426" spans="1:14" ht="225" hidden="1" x14ac:dyDescent="0.25">
       <c r="A426" s="5">
         <v>123</v>
       </c>
@@ -23964,7 +24265,7 @@
       <c r="M426" s="5"/>
       <c r="N426" s="5"/>
     </row>
-    <row r="427" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="427" spans="1:14" ht="225" hidden="1" x14ac:dyDescent="0.25">
       <c r="A427" s="5">
         <v>6</v>
       </c>
@@ -24064,7 +24365,7 @@
       <c r="M429" s="5"/>
       <c r="N429" s="5"/>
     </row>
-    <row r="430" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="430" spans="1:14" ht="225" hidden="1" x14ac:dyDescent="0.25">
       <c r="A430" s="5">
         <v>400</v>
       </c>
@@ -24098,7 +24399,7 @@
       <c r="M430" s="5"/>
       <c r="N430" s="5"/>
     </row>
-    <row r="431" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="431" spans="1:14" ht="285" hidden="1" x14ac:dyDescent="0.25">
       <c r="A431" s="5">
         <v>137</v>
       </c>
@@ -24132,7 +24433,7 @@
       <c r="M431" s="5"/>
       <c r="N431" s="5"/>
     </row>
-    <row r="432" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="432" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A432" s="5">
         <v>345</v>
       </c>
@@ -24268,7 +24569,7 @@
       <c r="M435" s="5"/>
       <c r="N435" s="5"/>
     </row>
-    <row r="436" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="436" spans="1:14" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A436" s="5">
         <v>502</v>
       </c>
@@ -24336,7 +24637,7 @@
       <c r="M437" s="5"/>
       <c r="N437" s="5"/>
     </row>
-    <row r="438" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="438" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A438" s="5">
         <v>295</v>
       </c>
@@ -24374,7 +24675,7 @@
       <c r="M438" s="5"/>
       <c r="N438" s="5"/>
     </row>
-    <row r="439" spans="1:14" ht="255" x14ac:dyDescent="0.25">
+    <row r="439" spans="1:14" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A439" s="5">
         <v>69</v>
       </c>
@@ -24476,7 +24777,7 @@
       <c r="M441" s="5"/>
       <c r="N441" s="5"/>
     </row>
-    <row r="442" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="442" spans="1:14" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A442" s="5">
         <v>111</v>
       </c>
@@ -24542,7 +24843,7 @@
       <c r="M443" s="5"/>
       <c r="N443" s="5"/>
     </row>
-    <row r="444" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="444" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A444" s="5">
         <v>110</v>
       </c>
@@ -24678,7 +24979,7 @@
       <c r="M447" s="5"/>
       <c r="N447" s="5"/>
     </row>
-    <row r="448" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="448" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A448" s="5">
         <v>512</v>
       </c>
@@ -24712,7 +25013,7 @@
       <c r="M448" s="5"/>
       <c r="N448" s="5"/>
     </row>
-    <row r="449" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="449" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A449" s="5">
         <v>76</v>
       </c>
@@ -24746,7 +25047,7 @@
       <c r="M449" s="5"/>
       <c r="N449" s="5"/>
     </row>
-    <row r="450" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="450" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A450" s="5">
         <v>191</v>
       </c>
@@ -24814,7 +25115,7 @@
       <c r="M451" s="5"/>
       <c r="N451" s="5"/>
     </row>
-    <row r="452" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="452" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A452" s="5">
         <v>86</v>
       </c>
@@ -24848,7 +25149,7 @@
       <c r="M452" s="5"/>
       <c r="N452" s="5"/>
     </row>
-    <row r="453" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="453" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A453" s="5">
         <v>49</v>
       </c>
@@ -24914,7 +25215,7 @@
       <c r="M454" s="5"/>
       <c r="N454" s="5"/>
     </row>
-    <row r="455" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="455" spans="1:14" ht="285" hidden="1" x14ac:dyDescent="0.25">
       <c r="A455" s="5">
         <v>112</v>
       </c>
@@ -24948,7 +25249,7 @@
       <c r="M455" s="5"/>
       <c r="N455" s="5"/>
     </row>
-    <row r="456" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+    <row r="456" spans="1:14" ht="240" hidden="1" x14ac:dyDescent="0.25">
       <c r="A456" s="5">
         <v>287</v>
       </c>
@@ -24986,7 +25287,7 @@
       <c r="M456" s="5"/>
       <c r="N456" s="5"/>
     </row>
-    <row r="457" spans="1:14" ht="75" x14ac:dyDescent="0.25">
+    <row r="457" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A457" s="5">
         <v>372</v>
       </c>
@@ -25024,7 +25325,7 @@
       <c r="M457" s="5"/>
       <c r="N457" s="5"/>
     </row>
-    <row r="458" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="458" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A458" s="5">
         <v>514</v>
       </c>
@@ -25130,7 +25431,7 @@
       <c r="M460" s="5"/>
       <c r="N460" s="5"/>
     </row>
-    <row r="461" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="461" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A461" s="5">
         <v>75</v>
       </c>
@@ -25164,7 +25465,7 @@
       <c r="M461" s="5"/>
       <c r="N461" s="5"/>
     </row>
-    <row r="462" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="462" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A462" s="5">
         <v>465</v>
       </c>
@@ -25198,7 +25499,7 @@
       <c r="M462" s="5"/>
       <c r="N462" s="5"/>
     </row>
-    <row r="463" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="463" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A463" s="5">
         <v>208</v>
       </c>
@@ -25232,7 +25533,7 @@
       <c r="M463" s="5"/>
       <c r="N463" s="5"/>
     </row>
-    <row r="464" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="464" spans="1:14" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A464" s="5">
         <v>376</v>
       </c>
@@ -25300,7 +25601,7 @@
       <c r="M465" s="5"/>
       <c r="N465" s="5"/>
     </row>
-    <row r="466" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="466" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A466" s="5">
         <v>515</v>
       </c>
@@ -25334,7 +25635,7 @@
       <c r="M466" s="5"/>
       <c r="N466" s="5"/>
     </row>
-    <row r="467" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="467" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A467" s="5">
         <v>220</v>
       </c>
@@ -25402,7 +25703,7 @@
       <c r="M468" s="5"/>
       <c r="N468" s="5"/>
     </row>
-    <row r="469" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="469" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A469" s="5">
         <v>488</v>
       </c>
@@ -25436,7 +25737,7 @@
       <c r="M469" s="5"/>
       <c r="N469" s="5"/>
     </row>
-    <row r="470" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="470" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A470" s="5">
         <v>126</v>
       </c>
@@ -25536,7 +25837,7 @@
       <c r="M472" s="5"/>
       <c r="N472" s="5"/>
     </row>
-    <row r="473" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="473" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A473" s="5">
         <v>485</v>
       </c>
@@ -25570,7 +25871,7 @@
       <c r="M473" s="5"/>
       <c r="N473" s="5"/>
     </row>
-    <row r="474" spans="1:14" ht="330" x14ac:dyDescent="0.25">
+    <row r="474" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A474" s="5">
         <v>46</v>
       </c>
@@ -25636,7 +25937,7 @@
       <c r="M475" s="5"/>
       <c r="N475" s="5"/>
     </row>
-    <row r="476" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="476" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A476" s="5">
         <v>324</v>
       </c>
@@ -25670,7 +25971,7 @@
       <c r="M476" s="5"/>
       <c r="N476" s="5"/>
     </row>
-    <row r="477" spans="1:14" ht="270" x14ac:dyDescent="0.25">
+    <row r="477" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A477" s="5">
         <v>505</v>
       </c>
@@ -25704,7 +26005,7 @@
       <c r="M477" s="5"/>
       <c r="N477" s="5"/>
     </row>
-    <row r="478" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="478" spans="1:14" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A478" s="5">
         <v>303</v>
       </c>
@@ -25738,7 +26039,7 @@
       <c r="M478" s="5"/>
       <c r="N478" s="5"/>
     </row>
-    <row r="479" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="479" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A479" s="5">
         <v>242</v>
       </c>
@@ -25772,7 +26073,7 @@
       <c r="M479" s="5"/>
       <c r="N479" s="5"/>
     </row>
-    <row r="480" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="480" spans="1:14" ht="225" hidden="1" x14ac:dyDescent="0.25">
       <c r="A480" s="5">
         <v>148</v>
       </c>
@@ -25806,7 +26107,7 @@
       <c r="M480" s="5"/>
       <c r="N480" s="5"/>
     </row>
-    <row r="481" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="481" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A481" s="5">
         <v>393</v>
       </c>
@@ -25874,7 +26175,7 @@
       <c r="M482" s="5"/>
       <c r="N482" s="5"/>
     </row>
-    <row r="483" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="483" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A483" s="5">
         <v>237</v>
       </c>
@@ -25908,7 +26209,7 @@
       <c r="M483" s="5"/>
       <c r="N483" s="5"/>
     </row>
-    <row r="484" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="484" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A484" s="5">
         <v>352</v>
       </c>
@@ -25980,7 +26281,7 @@
       <c r="M485" s="5"/>
       <c r="N485" s="5"/>
     </row>
-    <row r="486" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="486" spans="1:14" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A486" s="5">
         <v>55</v>
       </c>
@@ -26012,7 +26313,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="487" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="487" spans="1:14" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A487" s="5">
         <v>534</v>
       </c>
@@ -26050,7 +26351,7 @@
       <c r="M487" s="5"/>
       <c r="N487" s="5"/>
     </row>
-    <row r="488" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="488" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A488" s="5">
         <v>426</v>
       </c>
@@ -26084,7 +26385,7 @@
       <c r="M488" s="5"/>
       <c r="N488" s="5"/>
     </row>
-    <row r="489" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="489" spans="1:14" ht="90" x14ac:dyDescent="0.25">
       <c r="A489" s="5">
         <v>12</v>
       </c>
@@ -26105,8 +26406,12 @@
       <c r="H489" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="I489" s="6"/>
-      <c r="J489" s="6"/>
+      <c r="I489" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J489" s="6" t="s">
+        <v>2642</v>
+      </c>
       <c r="K489" s="5" t="s">
         <v>107</v>
       </c>
@@ -26116,7 +26421,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="490" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="490" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A490" s="5">
         <v>510</v>
       </c>
@@ -26150,7 +26455,7 @@
       <c r="M490" s="5"/>
       <c r="N490" s="5"/>
     </row>
-    <row r="491" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="491" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A491" s="5">
         <v>156</v>
       </c>
@@ -26358,7 +26663,7 @@
       <c r="M496" s="5"/>
       <c r="N496" s="5"/>
     </row>
-    <row r="497" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+    <row r="497" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A497" s="5">
         <v>292</v>
       </c>
@@ -26396,7 +26701,7 @@
       <c r="M497" s="5"/>
       <c r="N497" s="5"/>
     </row>
-    <row r="498" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="498" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A498" s="5">
         <v>380</v>
       </c>
@@ -26536,7 +26841,7 @@
       <c r="M501" s="5"/>
       <c r="N501" s="5"/>
     </row>
-    <row r="502" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="502" spans="1:14" ht="225" x14ac:dyDescent="0.25">
       <c r="A502" s="5">
         <v>316</v>
       </c>
@@ -26561,8 +26866,12 @@
       <c r="H502" s="6" t="s">
         <v>2821</v>
       </c>
-      <c r="I502" s="6"/>
-      <c r="J502" s="6"/>
+      <c r="I502" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J502" s="6" t="s">
+        <v>2578</v>
+      </c>
       <c r="K502" s="5" t="s">
         <v>1538</v>
       </c>
@@ -26570,7 +26879,7 @@
       <c r="M502" s="5"/>
       <c r="N502" s="5"/>
     </row>
-    <row r="503" spans="1:14" ht="105" x14ac:dyDescent="0.25">
+    <row r="503" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A503" s="5">
         <v>462</v>
       </c>
@@ -26604,7 +26913,7 @@
       <c r="M503" s="5"/>
       <c r="N503" s="5"/>
     </row>
-    <row r="504" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="504" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A504" s="5">
         <v>448</v>
       </c>
@@ -26672,7 +26981,7 @@
       <c r="M505" s="5"/>
       <c r="N505" s="5"/>
     </row>
-    <row r="506" spans="1:14" ht="135" x14ac:dyDescent="0.25">
+    <row r="506" spans="1:14" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A506" s="5">
         <v>489</v>
       </c>
@@ -26812,7 +27121,7 @@
       <c r="M509" s="5"/>
       <c r="N509" s="5"/>
     </row>
-    <row r="510" spans="1:14" ht="270" x14ac:dyDescent="0.25">
+    <row r="510" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A510" s="5">
         <v>114</v>
       </c>
@@ -26846,7 +27155,7 @@
       <c r="M510" s="5"/>
       <c r="N510" s="5"/>
     </row>
-    <row r="511" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="511" spans="1:14" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A511" s="5">
         <v>281</v>
       </c>
@@ -26880,7 +27189,7 @@
       <c r="M511" s="5"/>
       <c r="N511" s="5"/>
     </row>
-    <row r="512" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="512" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A512" s="5">
         <v>15</v>
       </c>
@@ -26916,7 +27225,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="513" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="513" spans="1:14" ht="150" x14ac:dyDescent="0.25">
       <c r="A513" s="5">
         <v>89</v>
       </c>
@@ -26941,8 +27250,12 @@
       <c r="H513" s="6" t="s">
         <v>2590</v>
       </c>
-      <c r="I513" s="6"/>
-      <c r="J513" s="6"/>
+      <c r="I513" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J513" s="6" t="s">
+        <v>2642</v>
+      </c>
       <c r="K513" s="5" t="s">
         <v>469</v>
       </c>
@@ -26950,7 +27263,7 @@
       <c r="M513" s="5"/>
       <c r="N513" s="5"/>
     </row>
-    <row r="514" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="514" spans="1:14" ht="225" hidden="1" x14ac:dyDescent="0.25">
       <c r="A514" s="5">
         <v>231</v>
       </c>
@@ -26988,7 +27301,7 @@
       <c r="M514" s="5"/>
       <c r="N514" s="5"/>
     </row>
-    <row r="515" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="515" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A515" s="5">
         <v>207</v>
       </c>
@@ -27022,7 +27335,7 @@
       <c r="M515" s="5"/>
       <c r="N515" s="5"/>
     </row>
-    <row r="516" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="516" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A516" s="5">
         <v>104</v>
       </c>
@@ -27158,7 +27471,7 @@
       <c r="M519" s="5"/>
       <c r="N519" s="5"/>
     </row>
-    <row r="520" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="520" spans="1:14" ht="255" hidden="1" x14ac:dyDescent="0.25">
       <c r="A520" s="5">
         <v>285</v>
       </c>
@@ -27192,7 +27505,7 @@
       <c r="M520" s="5"/>
       <c r="N520" s="5"/>
     </row>
-    <row r="521" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="521" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A521" s="5">
         <v>14</v>
       </c>
@@ -27213,8 +27526,12 @@
       <c r="H521" s="6" t="s">
         <v>2831</v>
       </c>
-      <c r="I521" s="6"/>
-      <c r="J521" s="6"/>
+      <c r="I521" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J521" s="6" t="s">
+        <v>2642</v>
+      </c>
       <c r="K521" s="5" t="s">
         <v>114</v>
       </c>
@@ -27292,7 +27609,7 @@
       <c r="M523" s="5"/>
       <c r="N523" s="5"/>
     </row>
-    <row r="524" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="524" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A524" s="5">
         <v>452</v>
       </c>
@@ -27453,8 +27770,12 @@
       <c r="H528" s="6" t="s">
         <v>2755</v>
       </c>
-      <c r="I528" s="6"/>
-      <c r="J528" s="6"/>
+      <c r="I528" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J528" s="6" t="s">
+        <v>2840</v>
+      </c>
       <c r="K528" s="5" t="s">
         <v>1108</v>
       </c>
@@ -27564,7 +27885,7 @@
       <c r="M531" s="5"/>
       <c r="N531" s="5"/>
     </row>
-    <row r="532" spans="1:14" ht="195" x14ac:dyDescent="0.25">
+    <row r="532" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A532" s="5">
         <v>183</v>
       </c>
@@ -27598,7 +27919,7 @@
       <c r="M532" s="5"/>
       <c r="N532" s="5"/>
     </row>
-    <row r="533" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="533" spans="1:14" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A533" s="5">
         <v>513</v>
       </c>
@@ -27632,7 +27953,7 @@
       <c r="M533" s="5"/>
       <c r="N533" s="5"/>
     </row>
-    <row r="534" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="534" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A534" s="5">
         <v>469</v>
       </c>
@@ -27666,7 +27987,7 @@
       <c r="M534" s="5"/>
       <c r="N534" s="5"/>
     </row>
-    <row r="535" spans="1:14" ht="210" x14ac:dyDescent="0.25">
+    <row r="535" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A535" s="5">
         <v>58</v>
       </c>
@@ -27698,7 +28019,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="536" spans="1:14" ht="225" x14ac:dyDescent="0.25">
+    <row r="536" spans="1:14" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A536" s="5">
         <v>486</v>
       </c>
@@ -27766,7 +28087,7 @@
       <c r="M537" s="5"/>
       <c r="N537" s="5"/>
     </row>
-    <row r="538" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="538" spans="1:14" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A538" s="5">
         <v>336</v>
       </c>
@@ -27834,7 +28155,7 @@
       <c r="M539" s="5"/>
       <c r="N539" s="5"/>
     </row>
-    <row r="540" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="540" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A540" s="5">
         <v>451</v>
       </c>
@@ -28004,7 +28325,7 @@
       <c r="M544" s="5"/>
       <c r="N544" s="5"/>
     </row>
-    <row r="545" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="545" spans="1:14" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A545" s="5">
         <v>402</v>
       </c>
@@ -28042,7 +28363,7 @@
       <c r="M545" s="5"/>
       <c r="N545" s="5"/>
     </row>
-    <row r="546" spans="1:14" ht="180" x14ac:dyDescent="0.25">
+    <row r="546" spans="1:14" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A546" s="5">
         <v>229</v>
       </c>
@@ -28080,7 +28401,7 @@
       <c r="M546" s="5"/>
       <c r="N546" s="5"/>
     </row>
-    <row r="547" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+    <row r="547" spans="1:14" ht="195" x14ac:dyDescent="0.25">
       <c r="A547" s="5">
         <v>478</v>
       </c>
@@ -28105,8 +28426,12 @@
       <c r="H547" s="6" t="s">
         <v>2716</v>
       </c>
-      <c r="I547" s="6"/>
-      <c r="J547" s="6"/>
+      <c r="I547" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J547" s="6" t="s">
+        <v>2841</v>
+      </c>
       <c r="K547" s="5" t="s">
         <v>2265</v>
       </c>
@@ -28154,6 +28479,23 @@
       <filters>
         <filter val="Include"/>
         <filter val="Maybe"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="8">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+    <filterColumn colId="9">
+      <filters>
+        <filter val="EC1"/>
+        <filter val="EC3"/>
+        <filter val="EC4"/>
+        <filter val="EC7"/>
+        <filter val="EC7 | Need Review"/>
+        <filter val="EC7 | Needs Review"/>
+        <filter val="Passed by Mahmoud"/>
+        <filter val="Passed by Mahmoud | Needs Review"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A6:N547">
@@ -28321,6 +28663,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="fdfc4d53-a3e2-4067-87fb-654f669f5f1a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100625AE263ADC950428ACD95DBF965DBE8" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="456165eecac37edca9453d0a31fd656e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="fdfc4d53-a3e2-4067-87fb-654f669f5f1a" xmlns:ns4="8dc15417-3e83-4528-b5fa-12604128870f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b29e677667ede315c277cdb9c6fc3957" ns3:_="" ns4:_="">
     <xsd:import namespace="fdfc4d53-a3e2-4067-87fb-654f669f5f1a"/>
@@ -28547,24 +28906,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7B8A44E-2D9C-4BAF-A96F-A4D70197AD60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="8dc15417-3e83-4528-b5fa-12604128870f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="fdfc4d53-a3e2-4067-87fb-654f669f5f1a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="fdfc4d53-a3e2-4067-87fb-654f669f5f1a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BBD265D-EBF0-49D9-879B-1C30F9F22B98}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13349CAC-6219-4077-91E4-D4A44901CDC2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -28581,29 +28948,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BBD265D-EBF0-49D9-879B-1C30F9F22B98}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7B8A44E-2D9C-4BAF-A96F-A4D70197AD60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="8dc15417-3e83-4528-b5fa-12604128870f"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="fdfc4d53-a3e2-4067-87fb-654f669f5f1a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
doc: README.md for Stage2 Work
</commit_message>
<xml_diff>
--- a/Reproducible Section/Step 4 - Stage 2 Screening/QCNN_HQCNN_Screening_Stage2_WIP.xlsx
+++ b/Reproducible Section/Step 4 - Stage 2 Screening/QCNN_HQCNN_Screening_Stage2_WIP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User1\Documents\GitHub\SLR\Reproducible Section\Step 4 - Stage 2 Screening\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3060A46-84A0-46FC-AEFC-F0CCC6FB8791}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4757DF3B-056D-473F-AEFA-B38B60E6F89D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -234,7 +234,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4567" uniqueCount="2844">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4571" uniqueCount="2847">
   <si>
     <t>IDENTIFICATION</t>
   </si>
@@ -8766,13 +8766,22 @@
   </si>
   <si>
     <t>Total in WIP List [Zotero]</t>
+  </si>
+  <si>
+    <t>Studies lacking experimental validation or quantitative evaluation of the proposed QCNN/HQCNN model.</t>
+  </si>
+  <si>
+    <t>EC9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  EC9</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -8798,11 +8807,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
     </font>
   </fonts>
   <fills count="5">
@@ -9271,7 +9275,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="44" customWidth="1"/>
@@ -9449,8 +9453,17 @@
         <v>2837</v>
       </c>
       <c r="B23">
-        <f>COUNTIFS(Screening!G2:G548,"Exclude",Screening!H2:H548,"EC7")</f>
-        <v>51</v>
+        <f>COUNTIFS(Screening!G2:G548,"Exclude",Screening!H2:H548,"EC8")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>2846</v>
+      </c>
+      <c r="B24">
+        <f>COUNTIFS(Screening!G3:G549,"Exclude",Screening!H3:H549,"EC9")</f>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -9579,6 +9592,15 @@
       <c r="B41">
         <f>COUNTIFS(Screening!I4:I550,"Exclude",Screening!J4:J550,"EC8")</f>
         <v>54</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>2846</v>
+      </c>
+      <c r="B42">
+        <f>COUNTIFS(Screening!I4:I550,"Exclude",Screening!J4:J550,"EC9")</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -28654,8 +28676,13 @@
         <v>2835</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="5"/>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>2845</v>
+      </c>
+      <c r="B17" t="s">
+        <v>2844</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -28663,23 +28690,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="fdfc4d53-a3e2-4067-87fb-654f669f5f1a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100625AE263ADC950428ACD95DBF965DBE8" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="456165eecac37edca9453d0a31fd656e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="fdfc4d53-a3e2-4067-87fb-654f669f5f1a" xmlns:ns4="8dc15417-3e83-4528-b5fa-12604128870f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b29e677667ede315c277cdb9c6fc3957" ns3:_="" ns4:_="">
     <xsd:import namespace="fdfc4d53-a3e2-4067-87fb-654f669f5f1a"/>
@@ -28906,32 +28916,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7B8A44E-2D9C-4BAF-A96F-A4D70197AD60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="8dc15417-3e83-4528-b5fa-12604128870f"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="fdfc4d53-a3e2-4067-87fb-654f669f5f1a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BBD265D-EBF0-49D9-879B-1C30F9F22B98}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="fdfc4d53-a3e2-4067-87fb-654f669f5f1a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13349CAC-6219-4077-91E4-D4A44901CDC2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -28948,4 +28950,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BBD265D-EBF0-49D9-879B-1C30F9F22B98}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7B8A44E-2D9C-4BAF-A96F-A4D70197AD60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="8dc15417-3e83-4528-b5fa-12604128870f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="fdfc4d53-a3e2-4067-87fb-654f669f5f1a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>